<commit_message>
Calibrate big-box categories in full calculator with new-store and listed-peer data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ke8h4Zgp7WmQ6H3JyfNM4g
</commit_message>
<xml_diff>
--- a/output/Kalkulator_Anggaran_Interior_Toko.xlsx
+++ b/output/Kalkulator_Anggaran_Interior_Toko.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="241">
   <si>
     <t xml:space="preserve">PETUNJUK PENGGUNAAN — Kalkulator Amplop Anggaran Interior Toko</t>
   </si>
@@ -211,6 +211,12 @@
     <t xml:space="preserve">• Semua angka di sheet Parameter adalah kisaran indikatif (Jabodetabek, kualitas menengah, ±2025–2026), hasil turunan asumsi industri umum — bukan data resmi atau milik merek tertentu.</t>
   </si>
   <si>
+    <t xml:space="preserve">• UPDATE: kategori 'Perlengkapan rumah &amp; perkakas' dan 'Furnitur &amp; dekorasi rumah' sudah dikalibrasi dengan data agregat toko baru dan laporan keuangan emiten sejenis (lihat catatan merah di sheet Parameter).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Jika memakai EBITDA dari laporan keuangan perusahaan: sejak PSAK 73 angka itu belum dikurangi sewa toko. Kurangi ±4–6% dari penjualan sebelum dimasukkan ke kolom EBITDA di sheet Parameter.</t>
+  </si>
+  <si>
     <t xml:space="preserve">• Gunakan sebagai titik awal diskusi. Validasi dengan penawaran kontraktor dan data aktual klien.</t>
   </si>
   <si>
@@ -433,7 +439,7 @@
     <t xml:space="preserve">EBITDA toko % (dari tabel)</t>
   </si>
   <si>
-    <t xml:space="preserve">Laba operasional toko sebelum penyusutan.</t>
+    <t xml:space="preserve">Laba operasional toko SETELAH sewa, sebelum penyusutan.</t>
   </si>
   <si>
     <t xml:space="preserve">Porsi interior dari total capex</t>
@@ -538,7 +544,7 @@
     <t xml:space="preserve">K maks</t>
   </si>
   <si>
-    <t xml:space="preserve">EBITDA toko %</t>
+    <t xml:space="preserve">EBITDA toko % (setelah sewa)</t>
   </si>
   <si>
     <t xml:space="preserve">Target payback capex (thn)</t>
@@ -592,16 +598,16 @@
     <t xml:space="preserve">Furnitur &amp; dekorasi rumah (big-box)</t>
   </si>
   <si>
-    <t xml:space="preserve">2.000–8.000 m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Showroom = alat jual; stok &amp; display besar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.500–5.000 m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stok sangat besar (puluhan ribu SKU) mengurangi ruang capex.</t>
+    <t xml:space="preserve">2.300–9.000 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIKALIBRASI: biaya = fit-out toko baru (data agregat internal, ±Rp 1,0 jt/m²). EBITDA belum ada data publik, dipakai 10% (konservatif).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.400–6.000 m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIKALIBRASI: biaya = fit-out toko baru (data agregat internal, ±Rp 1,2–1,4 jt/m²). EBITDA 13% = EBITDA emiten sejenis 2024–2025 (16,8–19,8%) dikurangi sewa ±5% (efek PSAK 73).</t>
   </si>
   <si>
     <t xml:space="preserve">Apotek / toko kesehatan</t>
@@ -626,6 +632,9 @@
   </si>
   <si>
     <t xml:space="preserve">K = anggaran interior ÷ penjualan setahun (kondisi toko sudah stabil). K diturunkan dari: (EBITDA% − biaya modal stok%) × target payback × porsi interior.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KALIBRASI (update): dua kategori big-box memakai data agregat toko baru (biaya fit-out per m²) dan laporan keuangan emiten ritel perlengkapan rumah di BEI 2024–2025. PENTING: sejak PSAK 73, EBITDA di laporan keuangan belum dikurangi sewa toko. Kurangi ±4–6% sebelum dipakai di sini. Kategori lain masih angka indikatif umum.</t>
   </si>
   <si>
     <t xml:space="preserve">TABEL 2 — Alokasi anggaran interior per elemen (% dari total)</t>
@@ -754,7 +763,7 @@
     <numFmt numFmtId="171" formatCode="0.0&quot; thn&quot;"/>
     <numFmt numFmtId="172" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -835,6 +844,14 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -946,7 +963,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1107,6 +1124,10 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1163,7 +1184,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1403,7 +1424,7 @@
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:C44"/>
+  <dimension ref="B1:C46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1680,7 +1701,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C43" s="2" t="s">
         <v>62</v>
       </c>
@@ -1688,6 +1709,16 @@
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C44" s="2" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C45" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C46" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1728,12 +1759,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
@@ -1743,21 +1774,21 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -1767,13 +1798,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
@@ -1781,13 +1812,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
@@ -1795,13 +1826,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="15" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>3000</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
@@ -1809,13 +1840,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="15" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>2500000</v>
+        <v>1200000</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -1823,13 +1854,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="15" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C10" s="18" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -1837,13 +1868,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -1851,13 +1882,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -1865,13 +1896,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -1879,13 +1910,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
@@ -1893,11 +1924,11 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -1905,7 +1936,7 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -1915,14 +1946,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="15" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C18" s="20" t="n">
         <f aca="false">C8*C9</f>
-        <v>7500000000</v>
+        <v>3600000000</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
@@ -1930,14 +1961,14 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C19" s="20" t="n">
         <f aca="false">C18*12</f>
-        <v>90000000000</v>
+        <v>43200000000</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -1945,14 +1976,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="15" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C20" s="21" t="n">
         <f aca="false">INDEX(Parameter!$B$6:$B$14,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
         <v>0.09</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
@@ -1960,14 +1991,14 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="15" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C21" s="21" t="n">
         <f aca="false">INDEX(Parameter!$C$6:$C$14,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
         <v>0.13</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
@@ -1982,7 +2013,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
@@ -1997,7 +2028,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -2005,14 +2036,14 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C24" s="21" t="n">
         <f aca="false">IF($C$15="",C20,$C$15*0.85)*C22*C23</f>
         <v>0.09</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
@@ -2020,14 +2051,14 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C25" s="21" t="n">
         <f aca="false">IF($C$15="",C21,$C$15*1.15)*C22*C23</f>
         <v>0.13</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -2035,7 +2066,7 @@
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -2045,25 +2076,25 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="23" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G28" s="23"/>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="24" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C29" s="21" t="n">
         <f aca="false">C24</f>
@@ -2071,20 +2102,20 @@
       </c>
       <c r="D29" s="25" t="n">
         <f aca="false">$C$19*C29</f>
-        <v>8100000000</v>
+        <v>3888000000</v>
       </c>
       <c r="E29" s="25" t="n">
         <f aca="false">IF($C$8&gt;0,D29/$C$8,0)</f>
-        <v>2700000</v>
+        <v>1296000</v>
       </c>
       <c r="F29" s="26" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G29" s="26"/>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="24" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C30" s="21" t="n">
         <f aca="false">AVERAGE(C24,C25)</f>
@@ -2092,20 +2123,20 @@
       </c>
       <c r="D30" s="25" t="n">
         <f aca="false">$C$19*C30</f>
-        <v>9900000000</v>
+        <v>4752000000</v>
       </c>
       <c r="E30" s="25" t="n">
         <f aca="false">IF($C$8&gt;0,D30/$C$8,0)</f>
-        <v>3300000</v>
+        <v>1584000</v>
       </c>
       <c r="F30" s="26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G30" s="26"/>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="24" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C31" s="21" t="n">
         <f aca="false">C25</f>
@@ -2113,20 +2144,20 @@
       </c>
       <c r="D31" s="25" t="n">
         <f aca="false">$C$19*C31</f>
-        <v>11700000000</v>
+        <v>5616000000</v>
       </c>
       <c r="E31" s="25" t="n">
         <f aca="false">IF($C$8&gt;0,D31/$C$8,0)</f>
-        <v>3900000</v>
+        <v>1872000</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G31" s="26"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -2136,14 +2167,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="15" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C34" s="22" t="n">
         <f aca="false">INDEX(Parameter!$B$45:$B$47,MATCH($C$11,Parameter!$A$45:$A$47,0))</f>
         <v>1</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -2151,7 +2182,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C35" s="22" t="n">
         <f aca="false">INDEX(Parameter!$B$51:$B$53,MATCH($C$12,Parameter!$A$51:$A$53,0))</f>
@@ -2164,7 +2195,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="15" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C36" s="22" t="n">
         <f aca="false">INDEX(Parameter!$B$57:$B$58,MATCH($C$13,Parameter!$A$57:$A$58,0))</f>
@@ -2177,14 +2208,14 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C37" s="20" t="n">
         <f aca="false">INDEX(Parameter!$G$6:$G$14,MATCH($C$7,Parameter!$A$6:$A$14,0))*C34*C35*C36</f>
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
@@ -2192,11 +2223,11 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C38" s="20" t="n">
         <f aca="false">INDEX(Parameter!$H$6:$H$14,MATCH($C$7,Parameter!$A$6:$A$14,0))*C34*C35*C36</f>
-        <v>4000000</v>
+        <v>1600000</v>
       </c>
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
@@ -2205,11 +2236,11 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="15" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C39" s="20" t="n">
         <f aca="false">E30</f>
-        <v>3300000</v>
+        <v>1584000</v>
       </c>
       <c r="D39" s="10"/>
       <c r="E39" s="10"/>
@@ -2218,7 +2249,7 @@
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="24" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C40" s="27" t="str">
         <f aca="false">IF(C39&gt;=C38,"LONGGAR — anggaran di atas biaya pasar. Ruang untuk konsep lebih kuat / material lebih baik.",IF(C39&gt;=C37,"SESUAI — anggaran berada di kisaran biaya pasar. Desain kualitas menengah aman.","TIDAK CUKUP — anggaran di bawah biaya pasar. Sederhanakan spesifikasi, kurangi area yang didesain, atau cek ulang target penjualan."))</f>
@@ -2231,7 +2262,7 @@
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
@@ -2241,14 +2272,14 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C43" s="21" t="n">
         <f aca="false">INDEX(Parameter!$D$6:$D$14,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E43" s="10"/>
       <c r="F43" s="10"/>
@@ -2256,14 +2287,14 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="15" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C44" s="21" t="n">
         <f aca="false">INDEX(Parameter!$E$6:$E$14,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
         <v>0.65</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
@@ -2271,14 +2302,14 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C45" s="20" t="n">
         <f aca="false">IF(C44&gt;0,D30/C44,0)</f>
-        <v>15230769230.7692</v>
+        <v>7310769230.76923</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E45" s="10"/>
       <c r="F45" s="10"/>
@@ -2286,14 +2317,14 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="15" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C46" s="20" t="n">
         <f aca="false">C19*C43</f>
-        <v>9000000000</v>
+        <v>5616000000</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E46" s="10"/>
       <c r="F46" s="10"/>
@@ -2301,14 +2332,14 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="15" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C47" s="28" t="n">
         <f aca="false">IF(C46&gt;0,C45/C46,0)</f>
-        <v>1.69230769230769</v>
+        <v>1.30177514792899</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E47" s="10"/>
       <c r="F47" s="10"/>
@@ -2316,14 +2347,14 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="15" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C48" s="29" t="n">
         <f aca="false">C10*0.5</f>
         <v>2.5</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E48" s="10"/>
       <c r="F48" s="10"/>
@@ -2331,7 +2362,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="24" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C49" s="30" t="str">
         <f aca="false">IF(C46&lt;=0,"Isi data proyek terlebih dahulu.",IF(C47&lt;=C48,"SEHAT — payback ≤ 50% masa sewa.",IF(C47&lt;=C10*0.7,"KETAT — payback 50–70% masa sewa. Pertimbangkan tingkat Basic/Standard.","BERISIKO — payback &gt; 70% masa sewa. Turunkan anggaran atau negosiasikan sewa lebih panjang.")))</f>
@@ -2344,7 +2375,7 @@
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
@@ -2354,27 +2385,27 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="23" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E52" s="23" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F52" s="23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G52" s="23" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="15" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C53" s="21" t="n">
         <f aca="false">INDEX(Parameter!$B$20:$B$28,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
@@ -2382,23 +2413,23 @@
       </c>
       <c r="D53" s="20" t="n">
         <f aca="false">$D$29*C53</f>
-        <v>3240000000</v>
+        <v>1555200000</v>
       </c>
       <c r="E53" s="31" t="n">
         <f aca="false">$D$30*C53</f>
-        <v>3960000000</v>
+        <v>1900800000</v>
       </c>
       <c r="F53" s="20" t="n">
         <f aca="false">$D$31*C53</f>
-        <v>4680000000</v>
+        <v>2246400000</v>
       </c>
       <c r="G53" s="32" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C54" s="21" t="n">
         <f aca="false">INDEX(Parameter!$C$20:$C$28,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
@@ -2406,23 +2437,23 @@
       </c>
       <c r="D54" s="20" t="n">
         <f aca="false">$D$29*C54</f>
-        <v>1377000000</v>
+        <v>660960000</v>
       </c>
       <c r="E54" s="31" t="n">
         <f aca="false">$D$30*C54</f>
-        <v>1683000000</v>
+        <v>807840000</v>
       </c>
       <c r="F54" s="20" t="n">
         <f aca="false">$D$31*C54</f>
-        <v>1989000000</v>
+        <v>954720000</v>
       </c>
       <c r="G54" s="32" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="15" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C55" s="21" t="n">
         <f aca="false">INDEX(Parameter!$D$20:$D$28,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
@@ -2430,23 +2461,23 @@
       </c>
       <c r="D55" s="20" t="n">
         <f aca="false">$D$29*C55</f>
-        <v>1377000000</v>
+        <v>660960000</v>
       </c>
       <c r="E55" s="31" t="n">
         <f aca="false">$D$30*C55</f>
-        <v>1683000000</v>
+        <v>807840000</v>
       </c>
       <c r="F55" s="20" t="n">
         <f aca="false">$D$31*C55</f>
-        <v>1989000000</v>
+        <v>954720000</v>
       </c>
       <c r="G55" s="32" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="15" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C56" s="21" t="n">
         <f aca="false">INDEX(Parameter!$E$20:$E$28,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
@@ -2454,23 +2485,23 @@
       </c>
       <c r="D56" s="20" t="n">
         <f aca="false">$D$29*C56</f>
-        <v>810000000</v>
+        <v>388800000</v>
       </c>
       <c r="E56" s="31" t="n">
         <f aca="false">$D$30*C56</f>
-        <v>990000000</v>
+        <v>475200000</v>
       </c>
       <c r="F56" s="20" t="n">
         <f aca="false">$D$31*C56</f>
-        <v>1170000000</v>
+        <v>561600000</v>
       </c>
       <c r="G56" s="32" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="15" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C57" s="21" t="n">
         <f aca="false">INDEX(Parameter!$F$20:$F$28,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
@@ -2478,23 +2509,23 @@
       </c>
       <c r="D57" s="20" t="n">
         <f aca="false">$D$29*C57</f>
-        <v>729000000</v>
+        <v>349920000</v>
       </c>
       <c r="E57" s="31" t="n">
         <f aca="false">$D$30*C57</f>
-        <v>891000000</v>
+        <v>427680000</v>
       </c>
       <c r="F57" s="20" t="n">
         <f aca="false">$D$31*C57</f>
-        <v>1053000000</v>
+        <v>505440000</v>
       </c>
       <c r="G57" s="32" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="15" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C58" s="21" t="n">
         <f aca="false">INDEX(Parameter!$G$20:$G$28,MATCH($C$7,Parameter!$A$6:$A$14,0))</f>
@@ -2502,23 +2533,23 @@
       </c>
       <c r="D58" s="20" t="n">
         <f aca="false">$D$29*C58</f>
-        <v>567000000</v>
+        <v>272160000</v>
       </c>
       <c r="E58" s="31" t="n">
         <f aca="false">$D$30*C58</f>
-        <v>693000000</v>
+        <v>332640000</v>
       </c>
       <c r="F58" s="20" t="n">
         <f aca="false">$D$31*C58</f>
-        <v>819000000</v>
+        <v>393120000</v>
       </c>
       <c r="G58" s="32" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="24" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C59" s="33" t="n">
         <f aca="false">SUM(C53:C58)</f>
@@ -2526,20 +2557,20 @@
       </c>
       <c r="D59" s="34" t="n">
         <f aca="false">SUM(D53:D58)</f>
-        <v>8100000000</v>
+        <v>3888000000</v>
       </c>
       <c r="E59" s="34" t="n">
         <f aca="false">SUM(E53:E58)</f>
-        <v>9900000000</v>
+        <v>4752000000</v>
       </c>
       <c r="F59" s="34" t="n">
         <f aca="false">SUM(F53:F58)</f>
-        <v>11700000000</v>
+        <v>5616000000</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="26" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C61" s="26"/>
       <c r="D61" s="26"/>
@@ -2681,12 +2712,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="35" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -2700,44 +2731,44 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="37" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G5" s="37" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="H5" s="37" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I5" s="37" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J5" s="37" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B6" s="19" t="n">
         <v>0.18</v>
@@ -2761,15 +2792,15 @@
         <v>8000000</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="J6" s="39" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B7" s="19" t="n">
         <v>0.2</v>
@@ -2793,15 +2824,15 @@
         <v>7000000</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="J7" s="39" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B8" s="19" t="n">
         <v>0.2</v>
@@ -2825,13 +2856,13 @@
         <v>6000000</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="J8" s="39"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B9" s="19" t="n">
         <v>0.2</v>
@@ -2855,15 +2886,15 @@
         <v>8000000</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="J9" s="39" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B10" s="19" t="n">
         <v>0.1</v>
@@ -2881,21 +2912,21 @@
         <v>3</v>
       </c>
       <c r="G10" s="17" t="n">
-        <v>2500000</v>
+        <v>800000</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>5000000</v>
+        <v>1300000</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="J10" s="39" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B11" s="19" t="n">
         <v>0.09</v>
@@ -2904,7 +2935,7 @@
         <v>0.13</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="E11" s="19" t="n">
         <v>0.65</v>
@@ -2913,21 +2944,21 @@
         <v>2.5</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="H11" s="17" t="n">
-        <v>4000000</v>
+        <v>1600000</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="J11" s="39" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B12" s="19" t="n">
         <v>0.04</v>
@@ -2951,13 +2982,13 @@
         <v>3000000</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="J12" s="39"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B13" s="19" t="n">
         <v>0.04</v>
@@ -2981,15 +3012,15 @@
         <v>3000000</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="J13" s="39" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B14" s="19" t="n">
         <v>0.04</v>
@@ -3013,15 +3044,15 @@
         <v>6000000</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="J14" s="39" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -3033,35 +3064,49 @@
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
     </row>
+    <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="40" t="s">
+        <v>203</v>
+      </c>
+      <c r="B16" s="40"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="40"/>
+    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="36" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="40" t="s">
-        <v>74</v>
+      <c r="A19" s="41" t="s">
+        <v>76</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D19" s="37" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F19" s="37" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G19" s="37" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H19" s="37" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3318,25 +3363,25 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="36" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="40" t="s">
-        <v>204</v>
-      </c>
-      <c r="B32" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="C32" s="41" t="s">
-        <v>206</v>
+      <c r="A32" s="41" t="s">
+        <v>207</v>
+      </c>
+      <c r="B32" s="41" t="s">
+        <v>208</v>
+      </c>
+      <c r="C32" s="42" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B33" s="42" t="n">
+      <c r="B33" s="43" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -3344,7 +3389,7 @@
       <c r="A34" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B34" s="42" t="n">
+      <c r="B34" s="43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3352,7 +3397,7 @@
       <c r="A35" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B35" s="42" t="n">
+      <c r="B35" s="43" t="n">
         <v>1.15</v>
       </c>
     </row>
@@ -3360,158 +3405,159 @@
       <c r="A36" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B36" s="42" t="n">
+      <c r="B36" s="43" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="36" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="41" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="40" t="s">
-        <v>204</v>
-      </c>
-      <c r="B39" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="C39" s="41" t="s">
+      <c r="B39" s="41" t="s">
         <v>208</v>
+      </c>
+      <c r="C39" s="42" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B40" s="42" t="n">
+        <v>95</v>
+      </c>
+      <c r="B40" s="43" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B41" s="42" t="n">
+        <v>212</v>
+      </c>
+      <c r="B41" s="43" t="n">
         <v>1.25</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="36" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="40" t="s">
-        <v>204</v>
-      </c>
-      <c r="B44" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="C44" s="41" t="s">
-        <v>211</v>
+      <c r="A44" s="41" t="s">
+        <v>207</v>
+      </c>
+      <c r="B44" s="41" t="s">
+        <v>208</v>
+      </c>
+      <c r="C44" s="42" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B45" s="42" t="n">
+        <v>86</v>
+      </c>
+      <c r="B45" s="43" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="B46" s="42" t="n">
+        <v>215</v>
+      </c>
+      <c r="B46" s="43" t="n">
         <v>0.85</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="B47" s="42" t="n">
+        <v>216</v>
+      </c>
+      <c r="B47" s="43" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="36" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="40" t="s">
-        <v>204</v>
-      </c>
-      <c r="B50" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="C50" s="41" t="s">
-        <v>215</v>
+      <c r="A50" s="41" t="s">
+        <v>207</v>
+      </c>
+      <c r="B50" s="41" t="s">
+        <v>208</v>
+      </c>
+      <c r="C50" s="42" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B51" s="42" t="n">
+        <v>89</v>
+      </c>
+      <c r="B51" s="43" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="B52" s="42" t="n">
+        <v>219</v>
+      </c>
+      <c r="B52" s="43" t="n">
         <v>1.15</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B53" s="42" t="n">
+        <v>220</v>
+      </c>
+      <c r="B53" s="43" t="n">
         <v>0.85</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="36" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="40" t="s">
-        <v>204</v>
-      </c>
-      <c r="B56" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="C56" s="41" t="s">
-        <v>219</v>
+      <c r="A56" s="41" t="s">
+        <v>207</v>
+      </c>
+      <c r="B56" s="41" t="s">
+        <v>208</v>
+      </c>
+      <c r="C56" s="42" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B57" s="42" t="n">
+        <v>92</v>
+      </c>
+      <c r="B57" s="43" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="B58" s="42" t="n">
+        <v>223</v>
+      </c>
+      <c r="B58" s="43" t="n">
         <v>0.85</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A16:J16"/>
   </mergeCells>
   <conditionalFormatting sqref="H20:H28">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
@@ -3554,12 +3600,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="35" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3574,93 +3620,93 @@
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="37" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D4" s="37" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E4" s="37" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F4" s="37" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="G4" s="37" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="H4" s="37" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I4" s="37" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="J4" s="37" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="K4" s="37" t="s">
-        <v>230</v>
-      </c>
-      <c r="M4" s="40" t="s">
-        <v>231</v>
-      </c>
-      <c r="N4" s="43" t="s">
-        <v>232</v>
-      </c>
-      <c r="O4" s="43" t="s">
         <v>233</v>
       </c>
-      <c r="P4" s="43" t="s">
+      <c r="M4" s="41" t="s">
         <v>234</v>
+      </c>
+      <c r="N4" s="44" t="s">
+        <v>235</v>
+      </c>
+      <c r="O4" s="44" t="s">
+        <v>236</v>
+      </c>
+      <c r="P4" s="44" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C5" s="18" t="n">
         <v>2025</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>2800</v>
+        <v>2400</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>2300000</v>
+        <v>1150000</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>8400000000</v>
+        <v>3360000000</v>
       </c>
       <c r="H5" s="20" t="n">
         <f aca="false">IF(OR(E5="",F5=""),"",E5*F5*12)</f>
-        <v>77280000000</v>
+        <v>33120000000</v>
       </c>
       <c r="I5" s="21" t="n">
         <f aca="false">IF(OR(G5="",H5="",H5=0),"",G5/H5)</f>
-        <v>0.108695652173913</v>
+        <v>0.101449275362319</v>
       </c>
       <c r="J5" s="20" t="n">
         <f aca="false">IF(OR(G5="",E5="",E5=0),"",G5/E5)</f>
-        <v>3000000</v>
+        <v>1400000</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="M5" s="5" t="str">
         <f aca="false">Parameter!A6</f>
         <v>Kafe / resto (F&amp;B)</v>
       </c>
-      <c r="N5" s="44" t="n">
+      <c r="N5" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M5,$I$5:$I$104,"&gt;0")</f>
         <v>0</v>
       </c>
@@ -3698,7 +3744,7 @@
         <f aca="false">Parameter!A7</f>
         <v>Fashion / aksesoris</v>
       </c>
-      <c r="N6" s="44" t="n">
+      <c r="N6" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M6,$I$5:$I$104,"&gt;0")</f>
         <v>0</v>
       </c>
@@ -3736,7 +3782,7 @@
         <f aca="false">Parameter!A8</f>
         <v>Salon</v>
       </c>
-      <c r="N7" s="44" t="n">
+      <c r="N7" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M7,$I$5:$I$104,"&gt;0")</f>
         <v>0</v>
       </c>
@@ -3774,7 +3820,7 @@
         <f aca="false">Parameter!A9</f>
         <v>Klinik kecantikan / kesehatan</v>
       </c>
-      <c r="N8" s="44" t="n">
+      <c r="N8" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M8,$I$5:$I$104,"&gt;0")</f>
         <v>0</v>
       </c>
@@ -3812,7 +3858,7 @@
         <f aca="false">Parameter!A10</f>
         <v>Furnitur &amp; dekorasi rumah (big-box)</v>
       </c>
-      <c r="N9" s="44" t="n">
+      <c r="N9" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M9,$I$5:$I$104,"&gt;0")</f>
         <v>0</v>
       </c>
@@ -3850,13 +3896,13 @@
         <f aca="false">Parameter!A11</f>
         <v>Perlengkapan rumah &amp; perkakas (big-box)</v>
       </c>
-      <c r="N10" s="44" t="n">
+      <c r="N10" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M10,$I$5:$I$104,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="O10" s="21" t="n">
         <f aca="false">IF(N10=0,"-",AVERAGEIFS($I$5:$I$104,$B$5:$B$104,M10,$I$5:$I$104,"&gt;0"))</f>
-        <v>0.108695652173913</v>
+        <v>0.101449275362319</v>
       </c>
       <c r="P10" s="21" t="n">
         <f aca="false">AVERAGE(Parameter!B11,Parameter!C11)</f>
@@ -3888,7 +3934,7 @@
         <f aca="false">Parameter!A12</f>
         <v>Apotek / toko kesehatan</v>
       </c>
-      <c r="N11" s="44" t="n">
+      <c r="N11" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M11,$I$5:$I$104,"&gt;0")</f>
         <v>0</v>
       </c>
@@ -3926,7 +3972,7 @@
         <f aca="false">Parameter!A13</f>
         <v>Minimarket / grocery</v>
       </c>
-      <c r="N12" s="44" t="n">
+      <c r="N12" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M12,$I$5:$I$104,"&gt;0")</f>
         <v>0</v>
       </c>
@@ -3964,7 +4010,7 @@
         <f aca="false">Parameter!A14</f>
         <v>Elektronik / gadget</v>
       </c>
-      <c r="N13" s="44" t="n">
+      <c r="N13" s="45" t="n">
         <f aca="false">COUNTIFS($B$5:$B$104,M13,$I$5:$I$104,"&gt;0")</f>
         <v>0</v>
       </c>
@@ -4021,7 +4067,7 @@
       </c>
       <c r="K15" s="4"/>
       <c r="M15" s="32" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>